<commit_message>
fix: gestion multi-CAV par PAV et PAV inactives (0 CAV)
- Les PAV avec nb_containers=0 sont marquées 'unavailable' automatiquement
- Les PAV avec >1 CAV conservent leur nb_containers réel (2, 3, 4, 6)
- QR codes générés uniquement pour les PAV actives
- Logs améliorés : total PAV, actives, inactives, total CAV (conteneurs)
- 209 PAV dont 197 actives (230 CAV) et 12 inactives

https://claude.ai/code/session_01FZ1s42Ui7SPkEDafW3ntCx
</commit_message>
<xml_diff>
--- a/Liste PAV.xlsx
+++ b/Liste PAV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliengonde/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9ACCC8DA-F1F9-0148-8EB1-AAAFA17E0D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCCBE1A7-265A-D94A-B7B7-F9EB8096BF00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1400" windowWidth="27640" windowHeight="16680" xr2:uid="{5DA664A1-39C7-A444-8818-CA5FC0068862}"/>
+    <workbookView xWindow="1500" yWindow="1380" windowWidth="27640" windowHeight="16680" xr2:uid="{5DA664A1-39C7-A444-8818-CA5FC0068862}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4762,7 +4762,6 @@
         <v>NOTRE-DAME-DE-BONDEVILLE - Rue des Bernardines (Devant les ateliers municipaux)</v>
       </c>
       <c r="B2" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C2" s="8" t="s">
@@ -4802,7 +4801,6 @@
         <v>DÉVILLE-LÈS-ROUEN - 8 Rue De Fontenelle</v>
       </c>
       <c r="B3" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C3" s="11" t="s">
@@ -4840,8 +4838,7 @@
         <v>DÉVILLE-LÈS-ROUEN - 34 Rue De Verdun</v>
       </c>
       <c r="B4" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>24</v>
@@ -4874,7 +4871,6 @@
         <v>ROUEN - 1 Avenue Jacques Chastellain (Ile Lacroix)</v>
       </c>
       <c r="B5" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -4914,7 +4910,6 @@
         <v>OISSEL - Rue Masson  (Place de la république)</v>
       </c>
       <c r="B6" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -4954,7 +4949,6 @@
         <v>OISSEL - 6 Avenue Du Général De Gaulle (Centre Commercial Saint Julien)</v>
       </c>
       <c r="B7" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -4994,7 +4988,6 @@
         <v>SOTTEVILLE-SOUS-LE-VAL - 2 Chemin des devises (Croisement avec Rue des canadiens)</v>
       </c>
       <c r="B8" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C8" s="11" t="s">
@@ -5034,7 +5027,6 @@
         <v>TOURVILLE-LA-RIVIÈRE - Rue Jean Jaures (Place de la Poste)</v>
       </c>
       <c r="B9" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C9" s="11" t="s">
@@ -5074,7 +5066,6 @@
         <v>CANTELEU - 36 Avenue de Versailles</v>
       </c>
       <c r="B10" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -5112,7 +5103,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 4 rue du Docteur Galouen</v>
       </c>
       <c r="B11" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C11" s="11" t="s">
@@ -5150,8 +5140,7 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 19 rue Marius Vallée (Face au gymnase)</v>
       </c>
       <c r="B12" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>66</v>
@@ -5186,7 +5175,6 @@
         <v>CANTELEU - 7 Rue Alexandre Dumas</v>
       </c>
       <c r="B13" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C13" s="11" t="s">
@@ -5224,7 +5212,6 @@
         <v>CANTELEU - 1 Avenue Charles Gounod (En face du collège)</v>
       </c>
       <c r="B14" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -5264,8 +5251,7 @@
         <v>LE PETIT-QUEVILLY - 57 avenue des Canadiens (Angle rue L. Antier)</v>
       </c>
       <c r="B15" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>78</v>
@@ -5300,8 +5286,7 @@
         <v>LE PETIT-QUEVILLY - 136 avenue des Martyrs de la Résistance (Angle rue du Maréchal Galliéni)</v>
       </c>
       <c r="B16" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>82</v>
@@ -5336,7 +5321,6 @@
         <v>PETIT-COURONNE - 44 Place Pierre Mendès France (Parking Coccinelle)</v>
       </c>
       <c r="B17" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C17" s="11" t="s">
@@ -5376,7 +5360,6 @@
         <v>PETIT-COURONNE - 220 Rue Du 14 Juillet (Croisement rue du Pommeret)</v>
       </c>
       <c r="B18" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -5416,7 +5399,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 103 rue Pierre Mendès-France (Parking Immeuble Habitat 76)</v>
       </c>
       <c r="B19" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C19" s="11" t="s">
@@ -5456,7 +5438,6 @@
         <v>AMFREVILLE-LA-MI-VOIE - 541 Chemin du Mesnil-Esnard (Parking de la crèche - Ecole Maternelle)</v>
       </c>
       <c r="B20" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C20" s="11" t="s">
@@ -5496,8 +5477,7 @@
         <v>BARENTIN - Centre commercial du Mesnil Roux (Parking Carrefour en face du Feu Vert)</v>
       </c>
       <c r="B21" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>107</v>
@@ -5534,7 +5514,6 @@
         <v>BONSECOURS - 23 Rue Camille Saint Saens (Parking du Stade des Hautes Haies)</v>
       </c>
       <c r="B22" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C22" s="8" t="s">
@@ -5574,7 +5553,6 @@
         <v>BOOS - 60 Impasse de la Grande Mare</v>
       </c>
       <c r="B23" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C23" s="8" t="s">
@@ -5612,7 +5590,6 @@
         <v>DARNÉTAL - 98 Rue Sadi Carnot (Face à la Mairie)</v>
       </c>
       <c r="B24" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
@@ -5652,7 +5629,6 @@
         <v>DARNÉTAL - 1 Rue de Préaux (Rond Point de la Girafe - Face à boulangerie)</v>
       </c>
       <c r="B25" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
@@ -5692,7 +5668,6 @@
         <v>DÉVILLE-LÈS-ROUEN - 51 Rue de la République (Devant Créapolis)</v>
       </c>
       <c r="B26" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
@@ -5732,7 +5707,6 @@
         <v>DÉVILLE-LÈS-ROUEN - 340 Route de Dieppe (Parking Salle communale (Mairie))</v>
       </c>
       <c r="B27" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
@@ -5772,8 +5746,7 @@
         <v>FRANQUEVILLE-SAINT-PIERRE - 962 Rue Pierre Curie (Cimetière)</v>
       </c>
       <c r="B28" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>145</v>
@@ -5812,7 +5785,6 @@
         <v>HÉNOUVILLE - 9 rue du Stade (Salle polyvalente - Ecole)</v>
       </c>
       <c r="B29" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C29" s="11" t="s">
@@ -5852,7 +5824,6 @@
         <v>HOUPPEVILLE - 140 Rue Louis Pasteur (Près des Jardins ouvriers)</v>
       </c>
       <c r="B30" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -5892,8 +5863,7 @@
         <v>ISNEAUVILLE - 3 Route de Dieppe (Parking Intermarché)</v>
       </c>
       <c r="B31" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>163</v>
@@ -5932,7 +5902,6 @@
         <v>MALAUNAY - 10 Rue Louis Lesouef (Parking face à Renault)</v>
       </c>
       <c r="B32" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C32" s="11" t="s">
@@ -5972,8 +5941,7 @@
         <v>LE MESNIL-ESNARD - 5 Rue des Perets (Parking de l'école)</v>
       </c>
       <c r="B33" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>175</v>
@@ -6012,8 +5980,7 @@
         <v>LE MESNIL-ESNARD - 3 Rue Gontran Pailhès (Carrefour Market)</v>
       </c>
       <c r="B34" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>181</v>
@@ -6052,8 +6019,7 @@
         <v>MONT-SAINT-AIGNAN - Centre Commercial La Vatine (Parking Carrefour)</v>
       </c>
       <c r="B35" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>186</v>
@@ -6092,7 +6058,6 @@
         <v>MONTVILLE - 693 rue des Reservoirs (Déchetterie - 9h30 / 11h45)</v>
       </c>
       <c r="B36" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C36" s="11" t="s">
@@ -6130,8 +6095,7 @@
         <v>MONTVILLE - 1 Sentier des Jumelles (Parking Intermarché)</v>
       </c>
       <c r="B37" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>198</v>
@@ -6168,7 +6132,6 @@
         <v>NOTRE-DAME-DE-BONDEVILLE - 90 rue des longs Vallons</v>
       </c>
       <c r="B38" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C38" s="8" t="s">
@@ -6206,7 +6169,6 @@
         <v>QUEVILLON - 31 Route de Belaitre (Parking Verger et Gite de Belaitre)</v>
       </c>
       <c r="B39" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C39" s="11" t="s">
@@ -6246,7 +6208,6 @@
         <v>QUINCAMPOIX - 11 Rue de Cailly (Parking du Cimetière)</v>
       </c>
       <c r="B40" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -6284,8 +6245,7 @@
         <v>ROUEN - 64 Boulevard d'Orléans (En face du Coccinelle)</v>
       </c>
       <c r="B41" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>218</v>
@@ -6320,7 +6280,6 @@
         <v>SAINT-AUBIN-EPINAY - 127 Rue de l'Eglise (Parking de l'école)</v>
       </c>
       <c r="B42" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C42" s="11" t="s">
@@ -6360,7 +6319,6 @@
         <v>SAINT-JACQUES-SUR-DARNÉTAL - 35 Rue de Verdun (Entre la Mairie et l'Eglise)</v>
       </c>
       <c r="B43" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C43" s="11" t="s">
@@ -6400,7 +6358,6 @@
         <v>SAINT-LÉGER-DU-BOURG-DENIS - 76 rue des Sources (Parking Mairie)</v>
       </c>
       <c r="B44" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C44" s="11" t="s">
@@ -6440,7 +6397,6 @@
         <v>SAINT-MARTIN-DE-BOSCHERVILLE - 62 Route de l'Abbaye (Au fond du parking)</v>
       </c>
       <c r="B45" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C45" s="11" t="s">
@@ -6480,7 +6436,6 @@
         <v>SAINT-MARTIN-DU-VIVIER - 1377 Route de la Vallée (Parking a coté de la Mairie)</v>
       </c>
       <c r="B46" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C46" s="11" t="s">
@@ -6520,7 +6475,6 @@
         <v>SAINT-PIERRE-DE-VARENGEVILLE - 240 Rue de la Paix (Parking du Cimetière)</v>
       </c>
       <c r="B47" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C47" s="11" t="s">
@@ -6560,8 +6514,7 @@
         <v>TOURVILLE-LA-RIVIÈRE - Avenue Gustave Picard (Parking Carrefour)</v>
       </c>
       <c r="B48" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>255</v>
@@ -6600,8 +6553,7 @@
         <v>LE TRAIT - 365 Rue Denis Papin (Parking Carrefour Market)</v>
       </c>
       <c r="B49" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" s="11" t="s">
         <v>259</v>
@@ -6640,7 +6592,6 @@
         <v>LA VAUPALIÈRE - 133 rue de l'Eglise (Parking en face de l'Espace WAPALLERIA)</v>
       </c>
       <c r="B50" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C50" s="11" t="s">
@@ -6678,7 +6629,6 @@
         <v>LE GRAND-QUEVILLY - 106 rue Paul Cezanne</v>
       </c>
       <c r="B51" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C51" s="11" t="s">
@@ -6716,7 +6666,6 @@
         <v>LA NEUVILLE-CHANT-D'OISEL - Rue du Froc aux Moines (Stade de Foot)</v>
       </c>
       <c r="B52" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C52" s="11" t="s">
@@ -6756,7 +6705,6 @@
         <v>SAINT-LÉGER-DU-BOURG-DENIS - 321 Rue des broches</v>
       </c>
       <c r="B53" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C53" s="11" t="s">
@@ -6794,7 +6742,6 @@
         <v>YAINVILLE - 1 Rue de la République (Allée derrière la pharmacie)</v>
       </c>
       <c r="B54" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -6834,7 +6781,6 @@
         <v>YMARE - Mairie (Pôle Déchets)</v>
       </c>
       <c r="B55" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C55" s="11" t="s">
@@ -6874,8 +6820,7 @@
         <v>ANNEVILLE-AMBOURVILLE - 2701 route de Bourg Achard (Déchetterie)</v>
       </c>
       <c r="B56" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>298</v>
@@ -6914,7 +6859,6 @@
         <v>BELBEUF - 8 rue des canadiens (Parking Salle Jacques Anquetil)</v>
       </c>
       <c r="B57" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C57" s="11" t="s">
@@ -6954,8 +6898,7 @@
         <v>BOIS-GUILLAUME - 2001 rue Herbeuse (Déchetterie - 9h / 12h - 14h / 17h30)</v>
       </c>
       <c r="B58" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>311</v>
@@ -6990,7 +6933,6 @@
         <v>BOOS - Rue des Canadiens (Déchetterie Boos - D91 vers Saint-Aubin-Celloville)</v>
       </c>
       <c r="B59" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C59" s="11" t="s">
@@ -7030,8 +6972,7 @@
         <v>DUCLAIR - 5 impasse du Maupas (Déchetterie Hameau les Monts 9h-12h / 13h30-17h30)</v>
       </c>
       <c r="B60" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" s="11" t="s">
         <v>320</v>
@@ -7070,7 +7011,6 @@
         <v>FONTAINE-SOUS-PRÉAUX - 81 Route de la Fontaine (Parking Salle des fêtes)</v>
       </c>
       <c r="B61" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C61" s="11" t="s">
@@ -7110,7 +7050,6 @@
         <v>QUÉVREVILLE-LA-POTERIE - Chemin du Vaudin (Parking Salle des fêtes)</v>
       </c>
       <c r="B62" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C62" s="11" t="s">
@@ -7150,7 +7089,6 @@
         <v>SAHURS - 3 Rue du Bas (Parking Place Maurice Alexandre)</v>
       </c>
       <c r="B63" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C63" s="11" t="s">
@@ -7190,7 +7128,6 @@
         <v>SAINT-PIERRE-DE-MANNEVILLE - 15 Route de Sahurs (Parking près de la mairie)</v>
       </c>
       <c r="B64" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C64" s="11" t="s">
@@ -7230,7 +7167,6 @@
         <v>LE TRAIT - Boulevard Industriel (Déchetterie LE TRAIT)</v>
       </c>
       <c r="B65" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C65" s="11" t="s">
@@ -7270,7 +7206,6 @@
         <v>VAL-DE-LA-HAYE - 2 Rue Henri Chivé</v>
       </c>
       <c r="B66" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C66" s="11" t="s">
@@ -7308,8 +7243,7 @@
         <v>LE PETIT-QUEVILLY - 438 Chemin du Gord (Déchetterie - 9h / 12h - 14h 17h00)</v>
       </c>
       <c r="B67" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" s="11" t="s">
         <v>359</v>
@@ -7348,7 +7282,6 @@
         <v>GRAND-COURONNE - 5 Allée de la Côté Mutel (Déchetterie - 9h / 12h - 14h - 17h30)</v>
       </c>
       <c r="B68" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C68" s="11" t="s">
@@ -7388,8 +7321,7 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 627 Rue de la Chaussée (Déchetterie)</v>
       </c>
       <c r="B69" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" s="11" t="s">
         <v>370</v>
@@ -7428,7 +7360,6 @@
         <v>CLÉON - Rue Marie-Louise et Raymond Boucher (Déchetterie de Cléon - 10h / 18h)</v>
       </c>
       <c r="B70" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C70" s="11" t="s">
@@ -7468,8 +7399,7 @@
         <v>SAINT-ÉTIENNE-DU-ROUVRAY - 47 Rue de Seine (Déchetterie - 9h / 12h - 14h / 17h)</v>
       </c>
       <c r="B71" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" s="11" t="s">
         <v>381</v>
@@ -7508,8 +7438,7 @@
         <v>ROUEN - 1 Quai du Pré aux loups (Dechetterie - 8h30 / 18h30)</v>
       </c>
       <c r="B72" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>387</v>
@@ -7548,7 +7477,6 @@
         <v>DARNÉTAL - 8 Sente de la Ravine (Déchetterie)</v>
       </c>
       <c r="B73" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C73" s="11" t="s">
@@ -7588,7 +7516,6 @@
         <v>DÉVILLE-LÈS-ROUEN - 18 Impasse Barbet (Déchetterie)</v>
       </c>
       <c r="B74" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C74" s="11" t="s">
@@ -7628,7 +7555,6 @@
         <v>SAINT-JEAN-DU-CARDONNAY - Côte de la Valette (Déchetterie de Maromme - 8h30 /18h30)</v>
       </c>
       <c r="B75" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C75" s="11" t="s">
@@ -7668,7 +7594,6 @@
         <v>HOUPPEVILLE - 86 rue de la Voix Maline (A coté de la colonne à verre)</v>
       </c>
       <c r="B76" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C76" s="11" t="s">
@@ -7708,7 +7633,6 @@
         <v>ISNEAUVILLE - 31 Rue André Le Nosle</v>
       </c>
       <c r="B77" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C77" s="11" t="s">
@@ -7746,7 +7670,6 @@
         <v>RONCHEROLLES-SUR-LE-VIVIER - 20 Impasse Des Prés Verts (Parking Centre De Loisirs Les Pépinières)</v>
       </c>
       <c r="B78" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C78" s="8" t="s">
@@ -7786,7 +7709,6 @@
         <v>DARNÉTAL - 37 Rue Edouard Branly</v>
       </c>
       <c r="B79" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C79" s="11" t="s">
@@ -7824,7 +7746,6 @@
         <v>DARNÉTAL - 33 Rue du Roule</v>
       </c>
       <c r="B80" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C80" s="11" t="s">
@@ -7862,7 +7783,6 @@
         <v>LES AUTHIEUX-SUR-LE-PORT-SAINT-OUEN - 260 rue du Docteur Gallouen (Parking de la salle des fêtes)</v>
       </c>
       <c r="B81" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C81" s="11" t="s">
@@ -7902,7 +7822,6 @@
         <v>HAUTOT-SUR-SEINE - 8 rue de l'Eglise (Place Poullard)</v>
       </c>
       <c r="B82" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C82" s="11" t="s">
@@ -7942,7 +7861,6 @@
         <v>LE GRAND-QUEVILLY - 26 Rue Michel Corroy (Place Du Québec)</v>
       </c>
       <c r="B83" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C83" s="11" t="s">
@@ -7982,7 +7900,6 @@
         <v>LE GRAND-QUEVILLY - 41 Avenue J. F. Kennedy</v>
       </c>
       <c r="B84" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C84" s="11" t="s">
@@ -8020,7 +7937,6 @@
         <v>LE GRAND-QUEVILLY - 132 Rue de la République (Centre Marx Dormoy)</v>
       </c>
       <c r="B85" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C85" s="11" t="s">
@@ -8060,7 +7976,6 @@
         <v>MOULINEAUX - 79 Chemin des Coquelicots</v>
       </c>
       <c r="B86" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C86" s="11" t="s">
@@ -8098,7 +8013,6 @@
         <v xml:space="preserve">LA BOUILLE - 111 Allée des Lauriers </v>
       </c>
       <c r="B87" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C87" s="11" t="s">
@@ -8136,7 +8050,6 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - 26 Rue de Freneuse (Croisement ruelle Arthus)</v>
       </c>
       <c r="B88" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C88" s="11" t="s">
@@ -8176,7 +8089,6 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 1049 Rue de la Villette</v>
       </c>
       <c r="B89" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C89" s="11" t="s">
@@ -8214,7 +8126,6 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 318 Rue Antoine de Saint Exupery</v>
       </c>
       <c r="B90" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C90" s="11" t="s">
@@ -8252,7 +8163,6 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 856 Rue Emile Zola</v>
       </c>
       <c r="B91" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C91" s="11" t="s">
@@ -8290,7 +8200,6 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 8 Rue Lenormand</v>
       </c>
       <c r="B92" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C92" s="11" t="s">
@@ -8328,7 +8237,6 @@
         <v>AMFREVILLE-LA-MI-VOIE - 25 rue François Mitterrand</v>
       </c>
       <c r="B93" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C93" s="11" t="s">
@@ -8366,7 +8274,6 @@
         <v>DARNÉTAL - 2 rue Edouard Branly</v>
       </c>
       <c r="B94" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C94" s="8" t="s">
@@ -8404,8 +8311,7 @@
         <v>DUCLAIR - 28 rue de Ronnenberg (Face au Relais Dellard - Parking de droite)</v>
       </c>
       <c r="B95" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C95" s="11" t="s">
         <v>495</v>
@@ -8444,7 +8350,6 @@
         <v>LA LONDE - 30 rue des Fusillés (Croisement rue Frete)</v>
       </c>
       <c r="B96" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C96" s="11" t="s">
@@ -8484,7 +8389,6 @@
         <v>GOUY - 28 rue du Poste (Suivre "Résidence Perelles" - Sur le parking)</v>
       </c>
       <c r="B97" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C97" s="11" t="s">
@@ -8524,7 +8428,6 @@
         <v>ELBEUF - 13 Rue de Rouen (D 938 sortie ELBEUF)</v>
       </c>
       <c r="B98" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C98" s="11" t="s">
@@ -8562,7 +8465,6 @@
         <v>ELBEUF - 26 Rue Leveillé</v>
       </c>
       <c r="B99" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C99" s="11" t="s">
@@ -8600,7 +8502,6 @@
         <v>ELBEUF - 2 rue Jean Jaures (Sous le pont Jean Jaurès)</v>
       </c>
       <c r="B100" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C100" s="11" t="s">
@@ -8640,7 +8541,6 @@
         <v>SAINT-PIERRE-LÈS-ELBEUF - 67 rue Galbois (Parking à coté des écoles)</v>
       </c>
       <c r="B101" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C101" s="11" t="s">
@@ -8680,8 +8580,7 @@
         <v>SAINT-PIERRE-LÈS-ELBEUF - Route de Pont de l'Arche (En face L'Auto E.Leclerc)</v>
       </c>
       <c r="B102" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>534</v>
@@ -8720,7 +8619,6 @@
         <v>SAINT-PIERRE-LÈS-ELBEUF - 625 rue du Puits Mérot (Parking Leader Price / Face à la mairie)</v>
       </c>
       <c r="B103" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C103" s="11" t="s">
@@ -8760,7 +8658,6 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - 20 Espace Foudriots (Derrière La Poste)</v>
       </c>
       <c r="B104" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C104" s="11" t="s">
@@ -8800,7 +8697,6 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - 5 rue Pierre Saint Georges (Gare de Saint Aubin)</v>
       </c>
       <c r="B105" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C105" s="11" t="s">
@@ -8840,7 +8736,6 @@
         <v>CLÉON - 83 rue Alain Colas (Parking Leader Price)</v>
       </c>
       <c r="B106" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C106" s="11" t="s">
@@ -8880,7 +8775,6 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - Rue du Docteur Villers (CHI - Parking usagers)</v>
       </c>
       <c r="B107" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C107" s="11" t="s">
@@ -8920,8 +8814,7 @@
         <v>CAUDEBEC-LÈS-ELBEUF - 67 Rue de Strasbourg (Place de l'Assemblée)</v>
       </c>
       <c r="B108" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C108" s="11" t="s">
         <v>564</v>
@@ -8960,7 +8853,6 @@
         <v>LA SAUSSAYE - 22 Route du Neubourg (Derrière le Manoir Saint-Nicolas)</v>
       </c>
       <c r="B109" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C109" s="11" t="s">
@@ -8998,8 +8890,7 @@
         <v>SAINT-PIERRE-DES-FLEURS - Route de Neuboug (Parking Cimetière)</v>
       </c>
       <c r="B110" s="13">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C110" s="8" t="s">
         <v>575</v>
@@ -9032,8 +8923,7 @@
         <v>SAINT-OUEN-DU-TILLEUL - 40 rue des Canadiens (Face à la Mairie)</v>
       </c>
       <c r="B111" s="13">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>579</v>
@@ -9070,7 +8960,6 @@
         <v>LA LONDE - 590 rue Adolphe Marie (Stade de Foot)</v>
       </c>
       <c r="B112" s="13">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C112" s="8" t="s">
@@ -9110,7 +8999,6 @@
         <v>ELBEUF - 7 Rue du Neubourg (Carrefour Market - Station Service)</v>
       </c>
       <c r="B113" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C113" s="11" t="s">
@@ -9150,7 +9038,6 @@
         <v>ORIVAL - 26 Rue de Rouen</v>
       </c>
       <c r="B114" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C114" s="11" t="s">
@@ -9188,8 +9075,7 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - CHI  rue du docteur Villers (entrée des urgences)</v>
       </c>
       <c r="B115" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C115" s="11" t="s">
         <v>599</v>
@@ -9224,7 +9110,6 @@
         <v>LE HOULME - 73 A rue du Général de Gaulle (Devant l'Association)</v>
       </c>
       <c r="B116" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C116" s="11" t="s">
@@ -9264,7 +9149,6 @@
         <v>FRENEUSE - 4 rue Côte aux Blancs</v>
       </c>
       <c r="B117" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C117" s="11" t="s">
@@ -9302,8 +9186,7 @@
         <v>BOURG-ACHARD - 510 Rue du Dr Duvrac (Parking Loic Gréaume)</v>
       </c>
       <c r="B118" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C118" s="11" t="s">
         <v>613</v>
@@ -9340,7 +9223,6 @@
         <v>LE GRAND-QUEVILLY - 18 Rue Maryse Bastié (Parking école Maryse Bastié)</v>
       </c>
       <c r="B119" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C119" s="11" t="s">
@@ -9380,7 +9262,6 @@
         <v>LE GRAND-QUEVILLY - 1 Rue Joseph-Jérome De Lalande (Parking)</v>
       </c>
       <c r="B120" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C120" s="11" t="s">
@@ -9420,7 +9301,6 @@
         <v>QUATREMARE - 3 route de Louviers</v>
       </c>
       <c r="B121" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C121" s="11" t="s">
@@ -9456,7 +9336,6 @@
         <v>ROMILLY-SUR-ANDELLE - 1674 rue Blingue</v>
       </c>
       <c r="B122" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C122" s="11" t="s">
@@ -9492,7 +9371,6 @@
         <v>LOUVIERS - 2 rue Saint-Jean (CHU - Dans l'enceinte de l'Hôpital - Parking)</v>
       </c>
       <c r="B123" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C123" s="11" t="s">
@@ -9530,7 +9408,6 @@
         <v>PITRES - 30 Rue de l'Eglise (Salle des fêtes)</v>
       </c>
       <c r="B124" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C124" s="11" t="s">
@@ -9568,7 +9445,6 @@
         <v>ROUEN - 72 rue de Martainville</v>
       </c>
       <c r="B125" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C125" s="11" t="s">
@@ -9606,7 +9482,6 @@
         <v>ROUEN - 27 Rue Verte (Gare)</v>
       </c>
       <c r="B126" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C126" s="11" t="s">
@@ -9646,7 +9521,6 @@
         <v>ROUEN - 35 rue Orbe (Près de Franprix)</v>
       </c>
       <c r="B127" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C127" s="11" t="s">
@@ -9686,7 +9560,6 @@
         <v>ROUEN - 25 rue de la Poterne (Entrée escalier Parking)</v>
       </c>
       <c r="B128" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C128" s="11" t="s">
@@ -9726,7 +9599,6 @@
         <v>ROUEN - 19 rue du Général Giraud</v>
       </c>
       <c r="B129" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C129" s="11" t="s">
@@ -9764,8 +9636,7 @@
         <v>ROUEN - 27 rue Saint-Sever (Cours Clémenceau)</v>
       </c>
       <c r="B130" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C130" s="11" t="s">
         <v>675</v>
@@ -9800,7 +9671,6 @@
         <v>ROUEN - 2 rue Blaise Pascal (Angle rue d'Elbeuf)</v>
       </c>
       <c r="B131" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C131" s="11" t="s">
@@ -9840,7 +9710,6 @@
         <v>ROUEN - 77 rue Méridienne (Angle Rue Octave Crutel)</v>
       </c>
       <c r="B132" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C132" s="11" t="s">
@@ -9880,7 +9749,6 @@
         <v>ROUEN - 9 rue Pierre Forfait (Angle Place de Lattre de Tassigny)</v>
       </c>
       <c r="B133" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C133" s="11" t="s">
@@ -9920,7 +9788,6 @@
         <v>SAINT-AUBIN-CELLOVILLE - 12 Rue de la Mairie  (Ruelle Atelier Municipal - Salle des Fêtes)</v>
       </c>
       <c r="B134" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C134" s="11" t="s">
@@ -9960,7 +9827,6 @@
         <v>ROUEN - 137 Route de Darnétal</v>
       </c>
       <c r="B135" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C135" s="11" t="s">
@@ -9998,7 +9864,6 @@
         <v>ROUEN - 2 Rue François Couperin (Parking Eglise Sainte-Claire)</v>
       </c>
       <c r="B136" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C136" s="11" t="s">
@@ -10038,7 +9903,6 @@
         <v>ROUEN - Rue du Chanoine Maubec (Angle Ferdinand Marrou - Derrière le Coccinelle)</v>
       </c>
       <c r="B137" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C137" s="11" t="s">
@@ -10078,7 +9942,6 @@
         <v>BAPEAUME-LÈS-ROUEN - 9021 Rue du Canal (Derrière la Station Service)</v>
       </c>
       <c r="B138" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C138" s="11" t="s">
@@ -10118,7 +9981,6 @@
         <v>DARNÉTAL - 10 rue aux Juifs</v>
       </c>
       <c r="B139" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C139" s="11" t="s">
@@ -10156,7 +10018,6 @@
         <v>MONTEROLIER - 1 Rue du Mesnil (Devant le terrain de tennis)</v>
       </c>
       <c r="B140" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C140" s="11" t="s">
@@ -10194,7 +10055,6 @@
         <v>NEUFCHATEL-EN-BRAY - 29 Impasse de la Gare (Face crèperie)</v>
       </c>
       <c r="B141" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C141" s="11" t="s">
@@ -10232,7 +10092,6 @@
         <v>ROCQUEMONT - 709 Grande Rue  (Côté Eglise)</v>
       </c>
       <c r="B142" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C142" s="11" t="s">
@@ -10270,7 +10129,6 @@
         <v>SOMMERY - 479 rue de la Gare (Parking Gare)</v>
       </c>
       <c r="B143" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C143" s="11" t="s">
@@ -10308,7 +10166,6 @@
         <v>BIHOREL - 212 Rue du Sansonnet  (Parking derrière Centre Commercial du Chapitre)</v>
       </c>
       <c r="B144" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C144" s="11" t="s">
@@ -10348,7 +10205,6 @@
         <v>BIHOREL - 15 Rue Philibert Caux (En face de l'école Ste Victrice)</v>
       </c>
       <c r="B145" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C145" s="11" t="s">
@@ -10388,7 +10244,6 @@
         <v>PONT-SAINT-PIERRE - 2 rue du Collège (Parking de la Piscine)</v>
       </c>
       <c r="B146" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C146" s="11" t="s">
@@ -10426,8 +10281,7 @@
         <v>INCARVILLE - 19 Rue des Prés (Parking Leclerc)</v>
       </c>
       <c r="B147" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C147" s="11" t="s">
         <v>764</v>
@@ -10464,7 +10318,6 @@
         <v>FONTAINE LE BOURG - 318 rue Delamare Deboutteville</v>
       </c>
       <c r="B148" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C148" s="11" t="s">
@@ -10500,7 +10353,6 @@
         <v>BIHOREL - 34 Rue de Verdun (Parking de la Piscine Transat)</v>
       </c>
       <c r="B149" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C149" s="11" t="s">
@@ -10540,7 +10392,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 59 Rue Pierre Bérégovoy (A coté de la colonne à verre)</v>
       </c>
       <c r="B150" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C150" s="11" t="s">
@@ -10580,7 +10431,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 36 rue Léon Salva (Angle rue Garibaldi)</v>
       </c>
       <c r="B151" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C151" s="11" t="s">
@@ -10620,7 +10470,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 30 avenue du 14 juillet (Parking Stade Sottevillais)</v>
       </c>
       <c r="B152" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C152" s="11" t="s">
@@ -10660,7 +10509,6 @@
         <v>MONT-SAINT-AIGNAN - 27 Boulevard André Siegfried</v>
       </c>
       <c r="B153" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C153" s="11" t="s">
@@ -10698,7 +10546,6 @@
         <v>SOTTEVILLE-LÈS-ROUEN - 4 Rue Paul Eluard (Hôpital Psychiatrique)</v>
       </c>
       <c r="B154" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C154" s="11" t="s">
@@ -10738,7 +10585,6 @@
         <v>LE PETIT-QUEVILLY - 87 rue Jean Macé (Croisement rue Francois Mitterand)</v>
       </c>
       <c r="B155" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C155" s="11" t="s">
@@ -10778,7 +10624,6 @@
         <v>LE PETIT-QUEVILLY - 152 rue Gambetta (Croisement rue Paul Langevin - Près école de musique)</v>
       </c>
       <c r="B156" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C156" s="11" t="s">
@@ -10818,7 +10663,6 @@
         <v>LE PETIT-QUEVILLY - 132 rue du Président Kennedy (Croisement rue de la République)</v>
       </c>
       <c r="B157" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C157" s="11" t="s">
@@ -10858,7 +10702,6 @@
         <v>MARTOT - 2 rue de l'Eure (Parking Eglise)</v>
       </c>
       <c r="B158" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C158" s="11" t="s">
@@ -10896,7 +10739,6 @@
         <v>SAINT-AUBIN-LÈS-ELBEUF - Rue du Docteur Villers (Entrée EHPAD)</v>
       </c>
       <c r="B159" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C159" s="11" t="s">
@@ -10934,7 +10776,6 @@
         <v>SAINT-ÉTIENNE-DU-ROUVRAY - 135 rue du Madrillet (Bâtiment AFPA)</v>
       </c>
       <c r="B160" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C160" s="11" t="s">
@@ -10974,7 +10815,6 @@
         <v>SAINT-MARTIN-DE-BOSCHERVILLE - 17 Chaussée Saint-Georges (Dechetterie)</v>
       </c>
       <c r="B161" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C161" s="11" t="s">
@@ -11014,7 +10854,6 @@
         <v>ROUEN - 49 Boulevard de Verdun (Au pied du Monumental)</v>
       </c>
       <c r="B162" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C162" s="11" t="s">
@@ -11054,7 +10893,6 @@
         <v>ROUEN - 19 rue Charles de Beaurepaire (Angle Côte de Neufchâtel)</v>
       </c>
       <c r="B163" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C163" s="11" t="s">
@@ -11094,7 +10932,6 @@
         <v>ROUEN - 14 Place du Boulingrin (Angle Rampe Beauvoisine)</v>
       </c>
       <c r="B164" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C164" s="11" t="s">
@@ -11134,7 +10971,6 @@
         <v>ROUEN - 86 Boulevard de l'Yser</v>
       </c>
       <c r="B165" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C165" s="11" t="s">
@@ -11172,7 +11008,6 @@
         <v>ROUEN - 44 Boulevard de la Marne (Angle Rampe Bouvreuil)</v>
       </c>
       <c r="B166" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C166" s="11" t="s">
@@ -11212,7 +11047,6 @@
         <v>ROUEN - 59 Rue Crevier (Angle rue d'Herbouville)</v>
       </c>
       <c r="B167" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C167" s="11" t="s">
@@ -11252,7 +11086,6 @@
         <v>ROUEN - 65 Rue Saint Maur (Angle rue Maladrerie)</v>
       </c>
       <c r="B168" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C168" s="11" t="s">
@@ -11292,8 +11125,7 @@
         <v>ROUEN - Rue Sénard (En face du 13 rue sénard)</v>
       </c>
       <c r="B169" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C169" s="11" t="s">
         <v>872</v>
@@ -11328,7 +11160,6 @@
         <v>ROUEN - 15 Rue Tabouret (Angle rue de la Cavée St Gervais)</v>
       </c>
       <c r="B170" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C170" s="11" t="s">
@@ -11368,7 +11199,6 @@
         <v>ROUEN - 3 Place Eglise Saint Gervais</v>
       </c>
       <c r="B171" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C171" s="11" t="s">
@@ -11406,7 +11236,6 @@
         <v>ROUEN - 23 rue Guillaume d'Estouteville</v>
       </c>
       <c r="B172" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C172" s="11" t="s">
@@ -11444,7 +11273,6 @@
         <v>ROUEN - 84 Rue du Renard (Ecole Achille Lefort)</v>
       </c>
       <c r="B173" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C173" s="11" t="s">
@@ -11484,7 +11312,6 @@
         <v>ROUEN - 43 Rue Stanislas Girardin (Angle rue A. Flaubert)</v>
       </c>
       <c r="B174" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C174" s="11" t="s">
@@ -11524,7 +11351,6 @@
         <v>ROUEN - 1 Place de la Madeleine (Angle rue Constantine)</v>
       </c>
       <c r="B175" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C175" s="11" t="s">
@@ -11564,7 +11390,6 @@
         <v>ROUEN - 29 Rue George d'Ambroise (Angle rue Duguay Trouin)</v>
       </c>
       <c r="B176" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C176" s="11" t="s">
@@ -11604,7 +11429,6 @@
         <v>ROUEN - 79 Rue Amédée Dormoy (A coté de l'entrée Intermarché)</v>
       </c>
       <c r="B177" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C177" s="11" t="s">
@@ -11644,7 +11468,6 @@
         <v>ROUEN - 145 Boulevard Jean Jaurès (Face au n°306)</v>
       </c>
       <c r="B178" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C178" s="11" t="s">
@@ -11684,7 +11507,6 @@
         <v>ROUEN - 2 rue du Loup</v>
       </c>
       <c r="B179" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C179" s="11" t="s">
@@ -11722,7 +11544,6 @@
         <v>MAROMME - 2 Rue de Binche (Parking école Delbos)</v>
       </c>
       <c r="B180" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C180" s="11" t="s">
@@ -11762,7 +11583,6 @@
         <v>MAROMME - 13 Route de Duclair (Parking Signa)</v>
       </c>
       <c r="B181" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C181" s="11" t="s">
@@ -11802,7 +11622,6 @@
         <v>JUMIÈGES - 752 Rue Alphonse Calais (Parking Camping-car)</v>
       </c>
       <c r="B182" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C182" s="11" t="s">
@@ -11842,7 +11661,6 @@
         <v>SAINT-PAËR - 119 Route de Duclair (Après le croisement Rue de l'église à coté des bacs à verre)</v>
       </c>
       <c r="B183" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C183" s="11" t="s">
@@ -11882,7 +11700,6 @@
         <v>BERVILLE-SUR-SEINE - 1061 rue du Village (Près de l'église)</v>
       </c>
       <c r="B184" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C184" s="11" t="s">
@@ -11922,7 +11739,6 @@
         <v>BARDOUVILLE - 300 rue de l’Ecole (En face du cimetière)</v>
       </c>
       <c r="B185" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C185" s="11" t="s">
@@ -11962,7 +11778,6 @@
         <v>SAINTE-MARGUERITE-SUR-DUCLAIR - 14 Route de Saint Paër (Parking)</v>
       </c>
       <c r="B186" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C186" s="11" t="s">
@@ -12002,7 +11817,6 @@
         <v>ARDOUVAL - 4 Rue des Bouleaux (Suivre panneau "Foyer des Jeunes")</v>
       </c>
       <c r="B187" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C187" s="11" t="s">
@@ -12040,7 +11854,6 @@
         <v>POMMEREVAL - 989 Route de l'Eglise</v>
       </c>
       <c r="B188" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C188" s="11" t="s">
@@ -12076,7 +11889,6 @@
         <v>BELLENCOMBRE - 2 bis Chemin du Cimetière</v>
       </c>
       <c r="B189" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C189" s="11" t="s">
@@ -12112,7 +11924,6 @@
         <v>COTTEVRARD - 77 Place de l'Eglise (En face de l'église - Parking au fond)</v>
       </c>
       <c r="B190" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C190" s="11" t="s">
@@ -12150,7 +11961,6 @@
         <v>BOSC LE HARD - 159 Rue des Forges</v>
       </c>
       <c r="B191" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C191" s="11" t="s">
@@ -12186,8 +11996,7 @@
         <v>ETOUTTEVILLE - 520 rue du Prieuré (Parking)</v>
       </c>
       <c r="B192" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C192" s="11" t="s">
         <v>989</v>
@@ -12224,7 +12033,6 @@
         <v>MOTTEVILLE - 156 Rue de la Gare (Face à la gare)</v>
       </c>
       <c r="B193" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C193" s="11" t="s">
@@ -12262,8 +12070,7 @@
         <v>FLAMANVILLE - 1 Rue de l'Eglise (Intersection Rue de l'Ecole)</v>
       </c>
       <c r="B194" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C194" s="11" t="s">
         <v>1000</v>
@@ -12300,7 +12107,6 @@
         <v>CIDEVILLE - 55 rue du Centre (A côté du garage et bacs verre)</v>
       </c>
       <c r="B195" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C195" s="11" t="s">
@@ -12337,8 +12143,7 @@
         <v>YERVILLE - 3 Place Bernard Alexandre</v>
       </c>
       <c r="B196" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C196" s="11" t="s">
         <v>1012</v>
@@ -12373,7 +12178,6 @@
         <v>VIBEUF - 25 rue de la Mare des Champs (Entrée parking communal)</v>
       </c>
       <c r="B197" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C197" s="11" t="s">
@@ -12411,7 +12215,6 @@
         <v>ROUEN - 229 Rue Saint Julien (Angle rue Parmentier)</v>
       </c>
       <c r="B198" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C198" s="11" t="s">
@@ -12451,8 +12254,7 @@
         <v>ROUEN - 238 Rue Saint Julien (Angle Rue Jacquard)</v>
       </c>
       <c r="B199" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C199" s="11" t="s">
         <v>1028</v>
@@ -12487,7 +12289,6 @@
         <v>ROUEN - 2 Rue du Mail (Angle Boulevard de l'Europe)</v>
       </c>
       <c r="B200" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C200" s="11" t="s">
@@ -12527,7 +12328,6 @@
         <v>ROUEN - 2 Rue Roger Bésus (Centre Charlotte Delbo)</v>
       </c>
       <c r="B201" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C201" s="11" t="s">
@@ -12567,7 +12367,6 @@
         <v>ROUEN - 46 Rue Desseaux (Proche bac verre)</v>
       </c>
       <c r="B202" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C202" s="11" t="s">
@@ -12607,7 +12406,6 @@
         <v>ROUEN - 11 Rue Antheaume (Résidence Vallon Saint Hilaire)</v>
       </c>
       <c r="B203" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C203" s="11" t="s">
@@ -12647,7 +12445,6 @@
         <v>ROUEN - 49 Rue de Bihorel (Angle rue Jouvenet)</v>
       </c>
       <c r="B204" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C204" s="11" t="s">
@@ -12687,8 +12484,7 @@
         <v>ROUEN - Avenue des Martyrs (Angle rue Linné)</v>
       </c>
       <c r="B205" s="7">
-        <f>COUNTA(#REF!)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C205" s="11" t="s">
         <v>1056</v>
@@ -12721,7 +12517,6 @@
         <v>ROUEN - 37 Rue de l'Enseigne Renaud (Angle Chemin de l'école Jules Ferry)</v>
       </c>
       <c r="B206" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C206" s="11" t="s">
@@ -12761,7 +12556,6 @@
         <v>ROUEN - 10 Rue Moise</v>
       </c>
       <c r="B207" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C207" s="11" t="s">
@@ -12799,7 +12593,6 @@
         <v>ROUEN - 41 Rue des Canadiens</v>
       </c>
       <c r="B208" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C208" s="11" t="s">
@@ -12837,7 +12630,6 @@
         <v>ROUEN - 5 place Saint Hilaire (Rond point Saint Hilaire)</v>
       </c>
       <c r="B209" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C209" s="11" t="s">
@@ -12877,7 +12669,6 @@
         <v>ROUEN - 53 rue Desseaux (Resto du Cœur)</v>
       </c>
       <c r="B210" s="7">
-        <f>COUNTA(#REF!)</f>
         <v>1</v>
       </c>
       <c r="C210" s="11" t="s">

</xml_diff>